<commit_message>
FK violation involving the users table returns a 401 instead of 500
</commit_message>
<xml_diff>
--- a/Document/Loyalty Program Logic.xlsx
+++ b/Document/Loyalty Program Logic.xlsx
@@ -20,6 +20,9 @@
     <sheet name="Members" sheetId="6" r:id="rId6"/>
     <sheet name="Invoice Log" sheetId="7" r:id="rId7"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId8"/>
+  </externalReferences>
   <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1472,6 +1475,70 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Settings"/>
+      <sheetName val="Bill Calculator"/>
+      <sheetName val="projections"/>
+      <sheetName val="Revenue Impact"/>
+      <sheetName val="Portfolio Tracker"/>
+      <sheetName val="Members"/>
+      <sheetName val="Invoice Log"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="16">
+          <cell r="B16">
+            <v>1</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="B31">
+            <v>2000</v>
+          </cell>
+          <cell r="C31">
+            <v>5000</v>
+          </cell>
+          <cell r="D31">
+            <v>10000</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="B32">
+            <v>0.05</v>
+          </cell>
+          <cell r="C32">
+            <v>0.1</v>
+          </cell>
+          <cell r="D32">
+            <v>0.15</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="B33">
+            <v>100</v>
+          </cell>
+          <cell r="C33">
+            <v>200</v>
+          </cell>
+          <cell r="D33">
+            <v>300</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2252,62 +2319,185 @@
         <v>1</v>
       </c>
       <c r="B9" s="31"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="41"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="72"/>
-      <c r="G9" s="73"/>
-      <c r="H9" s="78"/>
-      <c r="I9" s="72"/>
-      <c r="J9" s="74"/>
+      <c r="C9" s="40">
+        <v>1000000</v>
+      </c>
+      <c r="D9" s="41">
+        <f t="shared" ref="D9:D15" si="0">IF(C9="","",C9*$E$6)</f>
+        <v>80000</v>
+      </c>
+      <c r="E9" s="41">
+        <f t="shared" ref="E9:E15" si="1">IF(C9="","",C9-D9)</f>
+        <v>920000</v>
+      </c>
+      <c r="F9" s="72">
+        <f>IF(C9="","",(C9/1000*[1]Settings!$B$16*$H$6)+MAX(0,MIN(G9+(C9/1000*[1]Settings!$B$16*$H$6),[1]Settings!$C$31)-MAX(G9,[1]Settings!$B$31))*[1]Settings!$B$32+MAX(0,MIN(G9+(C9/1000*[1]Settings!$B$16*$H$6),[1]Settings!$D$31)-MAX(G9,[1]Settings!$C$31))*[1]Settings!$C$32+MAX(0,(G9+(C9/1000*[1]Settings!$B$16*$H$6))-MAX(G9,[1]Settings!$D$31))*[1]Settings!$D$32)</f>
+        <v>1000</v>
+      </c>
+      <c r="G9" s="73">
+        <f>IF(C9="","",0)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="78">
+        <f>IF(OR(C9="",C9=0),"",(F9-(C9/1000*[1]Settings!$B$16*$H$6))/(C9/1000*[1]Settings!$B$16*$H$6))</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="72">
+        <f>IF(C9="","",IF(AND(G9&lt;[1]Settings!$B$31,(G9+F9)&gt;=[1]Settings!$B$31),[1]Settings!$B$33,0)+IF(AND(G9&lt;[1]Settings!$C$31,(G9+F9)&gt;=[1]Settings!$C$31),[1]Settings!$C$33,0)+IF(AND(G9&lt;[1]Settings!$D$31,(G9+F9)&gt;=[1]Settings!$D$31),[1]Settings!$D$33,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="74">
+        <f>IF(C9="","",F9+I9)</f>
+        <v>1000</v>
+      </c>
     </row>
     <row r="10" spans="1:10" ht="19.5" customHeight="1">
       <c r="A10" s="35">
         <v>2</v>
       </c>
       <c r="B10" s="31"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="G10" s="73"/>
-      <c r="I10" s="72"/>
-      <c r="J10" s="74"/>
+      <c r="C10" s="40">
+        <v>100000</v>
+      </c>
+      <c r="D10" s="41">
+        <f t="shared" si="0"/>
+        <v>8000</v>
+      </c>
+      <c r="E10" s="41">
+        <f t="shared" si="1"/>
+        <v>92000</v>
+      </c>
+      <c r="F10">
+        <f>IF(C10="","",(C10/1000*[1]Settings!$B$16*$H$6)+MAX(0,MIN(G10+(C10/1000*[1]Settings!$B$16*$H$6),[1]Settings!$C$31)-MAX(G10,[1]Settings!$B$31))*[1]Settings!$B$32+MAX(0,MIN(G10+(C10/1000*[1]Settings!$B$16*$H$6),[1]Settings!$D$31)-MAX(G10,[1]Settings!$C$31))*[1]Settings!$C$32+MAX(0,(G10+(C10/1000*[1]Settings!$B$16*$H$6))-MAX(G10,[1]Settings!$D$31))*[1]Settings!$D$32)</f>
+        <v>100</v>
+      </c>
+      <c r="G10" s="73">
+        <f>IF(C10="","",SUM($J$9:J9))</f>
+        <v>1000</v>
+      </c>
+      <c r="H10">
+        <f>IF(OR(C10="",C10=0),"",(F10-(C10/1000*[1]Settings!$B$16*$H$6))/(C10/1000*[1]Settings!$B$16*$H$6))</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="72">
+        <f>IF(C10="","",IF(AND(G10&lt;[1]Settings!$B$31,(G10+F10)&gt;=[1]Settings!$B$31),[1]Settings!$B$33,0)+IF(AND(G10&lt;[1]Settings!$C$31,(G10+F10)&gt;=[1]Settings!$C$31),[1]Settings!$C$33,0)+IF(AND(G10&lt;[1]Settings!$D$31,(G10+F10)&gt;=[1]Settings!$D$31),[1]Settings!$D$33,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="74">
+        <f t="shared" ref="J10:J15" si="2">IF(C10="","",F10+I10)</f>
+        <v>100</v>
+      </c>
     </row>
     <row r="11" spans="1:10" ht="19.5" customHeight="1">
       <c r="A11" s="35">
         <v>3</v>
       </c>
       <c r="B11" s="31"/>
-      <c r="C11" s="40"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="41"/>
-      <c r="G11" s="73"/>
-      <c r="I11" s="72"/>
-      <c r="J11" s="74"/>
+      <c r="C11" s="40">
+        <v>2500000</v>
+      </c>
+      <c r="D11" s="41">
+        <f t="shared" si="0"/>
+        <v>200000</v>
+      </c>
+      <c r="E11" s="41">
+        <f t="shared" si="1"/>
+        <v>2300000</v>
+      </c>
+      <c r="F11">
+        <f>IF(C11="","",(C11/1000*[1]Settings!$B$16*$H$6)+MAX(0,MIN(G11+(C11/1000*[1]Settings!$B$16*$H$6),[1]Settings!$C$31)-MAX(G11,[1]Settings!$B$31))*[1]Settings!$B$32+MAX(0,MIN(G11+(C11/1000*[1]Settings!$B$16*$H$6),[1]Settings!$D$31)-MAX(G11,[1]Settings!$C$31))*[1]Settings!$C$32+MAX(0,(G11+(C11/1000*[1]Settings!$B$16*$H$6))-MAX(G11,[1]Settings!$D$31))*[1]Settings!$D$32)</f>
+        <v>2580</v>
+      </c>
+      <c r="G11" s="73">
+        <f>IF(C11="","",SUM($J$9:J10))</f>
+        <v>1100</v>
+      </c>
+      <c r="H11">
+        <f>IF(OR(C11="",C11=0),"",(F11-(C11/1000*[1]Settings!$B$16*$H$6))/(C11/1000*[1]Settings!$B$16*$H$6))</f>
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="I11" s="72">
+        <f>IF(C11="","",IF(AND(G11&lt;[1]Settings!$B$31,(G11+F11)&gt;=[1]Settings!$B$31),[1]Settings!$B$33,0)+IF(AND(G11&lt;[1]Settings!$C$31,(G11+F11)&gt;=[1]Settings!$C$31),[1]Settings!$C$33,0)+IF(AND(G11&lt;[1]Settings!$D$31,(G11+F11)&gt;=[1]Settings!$D$31),[1]Settings!$D$33,0))</f>
+        <v>100</v>
+      </c>
+      <c r="J11" s="74">
+        <f t="shared" si="2"/>
+        <v>2680</v>
+      </c>
     </row>
     <row r="12" spans="1:10" ht="19.5" customHeight="1">
       <c r="A12" s="35">
         <v>4</v>
       </c>
       <c r="B12" s="31"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="G12" s="73"/>
-      <c r="I12" s="72"/>
-      <c r="J12" s="74"/>
+      <c r="C12" s="40">
+        <v>600000</v>
+      </c>
+      <c r="D12" s="41">
+        <f t="shared" si="0"/>
+        <v>48000</v>
+      </c>
+      <c r="E12" s="41">
+        <f t="shared" si="1"/>
+        <v>552000</v>
+      </c>
+      <c r="F12">
+        <f>IF(C12="","",(C12/1000*[1]Settings!$B$16*$H$6)+MAX(0,MIN(G12+(C12/1000*[1]Settings!$B$16*$H$6),[1]Settings!$C$31)-MAX(G12,[1]Settings!$B$31))*[1]Settings!$B$32+MAX(0,MIN(G12+(C12/1000*[1]Settings!$B$16*$H$6),[1]Settings!$D$31)-MAX(G12,[1]Settings!$C$31))*[1]Settings!$C$32+MAX(0,(G12+(C12/1000*[1]Settings!$B$16*$H$6))-MAX(G12,[1]Settings!$D$31))*[1]Settings!$D$32)</f>
+        <v>630</v>
+      </c>
+      <c r="G12" s="73">
+        <f>IF(C12="","",SUM($J$9:J11))</f>
+        <v>3780</v>
+      </c>
+      <c r="H12">
+        <f>IF(OR(C12="",C12=0),"",(F12-(C12/1000*[1]Settings!$B$16*$H$6))/(C12/1000*[1]Settings!$B$16*$H$6))</f>
+        <v>0.05</v>
+      </c>
+      <c r="I12" s="72">
+        <f>IF(C12="","",IF(AND(G12&lt;[1]Settings!$B$31,(G12+F12)&gt;=[1]Settings!$B$31),[1]Settings!$B$33,0)+IF(AND(G12&lt;[1]Settings!$C$31,(G12+F12)&gt;=[1]Settings!$C$31),[1]Settings!$C$33,0)+IF(AND(G12&lt;[1]Settings!$D$31,(G12+F12)&gt;=[1]Settings!$D$31),[1]Settings!$D$33,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="74">
+        <f t="shared" si="2"/>
+        <v>630</v>
+      </c>
     </row>
     <row r="13" spans="1:10" ht="19.5" customHeight="1">
       <c r="A13" s="35">
         <v>5</v>
       </c>
       <c r="B13" s="31"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="G13" s="73"/>
-      <c r="I13" s="72"/>
-      <c r="J13" s="74"/>
+      <c r="C13" s="40">
+        <v>7500000</v>
+      </c>
+      <c r="D13" s="41">
+        <f t="shared" si="0"/>
+        <v>600000</v>
+      </c>
+      <c r="E13" s="41">
+        <f t="shared" si="1"/>
+        <v>6900000</v>
+      </c>
+      <c r="F13">
+        <f>IF(C13="","",(C13/1000*[1]Settings!$B$16*$H$6)+MAX(0,MIN(G13+(C13/1000*[1]Settings!$B$16*$H$6),[1]Settings!$C$31)-MAX(G13,[1]Settings!$B$31))*[1]Settings!$B$32+MAX(0,MIN(G13+(C13/1000*[1]Settings!$B$16*$H$6),[1]Settings!$D$31)-MAX(G13,[1]Settings!$C$31))*[1]Settings!$C$32+MAX(0,(G13+(C13/1000*[1]Settings!$B$16*$H$6))-MAX(G13,[1]Settings!$D$31))*[1]Settings!$D$32)</f>
+        <v>8316</v>
+      </c>
+      <c r="G13" s="73">
+        <f>IF(C13="","",SUM($J$9:J12))</f>
+        <v>4410</v>
+      </c>
+      <c r="H13">
+        <f>IF(OR(C13="",C13=0),"",(F13-(C13/1000*[1]Settings!$B$16*$H$6))/(C13/1000*[1]Settings!$B$16*$H$6))</f>
+        <v>0.10879999999999999</v>
+      </c>
+      <c r="I13" s="72">
+        <f>IF(C13="","",IF(AND(G13&lt;[1]Settings!$B$31,(G13+F13)&gt;=[1]Settings!$B$31),[1]Settings!$B$33,0)+IF(AND(G13&lt;[1]Settings!$C$31,(G13+F13)&gt;=[1]Settings!$C$31),[1]Settings!$C$33,0)+IF(AND(G13&lt;[1]Settings!$D$31,(G13+F13)&gt;=[1]Settings!$D$31),[1]Settings!$D$33,0))</f>
+        <v>500</v>
+      </c>
+      <c r="J13" s="74">
+        <f t="shared" si="2"/>
+        <v>8816</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="19.5" customHeight="1">
       <c r="A14" s="35">
@@ -2318,32 +2508,32 @@
         <v>7000000</v>
       </c>
       <c r="D14" s="41">
-        <f t="shared" ref="D9:D40" si="0">IF(C14="","",C14*$E$6)</f>
+        <f t="shared" si="0"/>
         <v>560000</v>
       </c>
       <c r="E14" s="41">
-        <f t="shared" ref="E9:E40" si="1">IF(C14="","",C14-D14)</f>
+        <f t="shared" si="1"/>
         <v>6440000</v>
       </c>
       <c r="F14">
-        <f>IF(C14="","",(C14/1000*Settings!$B$16*$H$6)+MAX(0,MIN(G14+(C14/1000*Settings!$B$16*$H$6),Settings!$C$31)-MAX(G14,Settings!$B$31))*Settings!$B$32+MAX(0,MIN(G14+(C14/1000*Settings!$B$16*$H$6),Settings!$D$31)-MAX(G14,Settings!$C$31))*Settings!$C$32+MAX(0,(G14+(C14/1000*Settings!$B$16*$H$6))-MAX(G14,Settings!$D$31))*Settings!$D$32)</f>
-        <v>7350</v>
+        <f>IF(C14="","",(C14/1000*[1]Settings!$B$16*$H$6)+MAX(0,MIN(G14+(C14/1000*[1]Settings!$B$16*$H$6),[1]Settings!$C$31)-MAX(G14,[1]Settings!$B$31))*[1]Settings!$B$32+MAX(0,MIN(G14+(C14/1000*[1]Settings!$B$16*$H$6),[1]Settings!$D$31)-MAX(G14,[1]Settings!$C$31))*[1]Settings!$C$32+MAX(0,(G14+(C14/1000*[1]Settings!$B$16*$H$6))-MAX(G14,[1]Settings!$D$31))*[1]Settings!$D$32)</f>
+        <v>8050</v>
       </c>
       <c r="G14" s="73">
         <f>IF(C14="","",SUM($J$9:J13))</f>
-        <v>0</v>
+        <v>13226</v>
       </c>
       <c r="H14">
-        <f>IF(OR(C14="",C14=0),"",(F14-(C14/1000*Settings!$B$16*$H$6))/(C14/1000*Settings!$B$16*$H$6))</f>
-        <v>0.05</v>
+        <f>IF(OR(C14="",C14=0),"",(F14-(C14/1000*[1]Settings!$B$16*$H$6))/(C14/1000*[1]Settings!$B$16*$H$6))</f>
+        <v>0.15</v>
       </c>
       <c r="I14" s="72">
-        <f>IF(C14="","",IF(AND(G14&lt;Settings!$B$31,(G14+F14)&gt;=Settings!$B$31),Settings!$B$33,0)+IF(AND(G14&lt;Settings!$C$31,(G14+F14)&gt;=Settings!$C$31),Settings!$C$33,0)+IF(AND(G14&lt;Settings!$D$31,(G14+F14)&gt;=Settings!$D$31),Settings!$D$33,0))</f>
-        <v>300</v>
+        <f>IF(C14="","",IF(AND(G14&lt;[1]Settings!$B$31,(G14+F14)&gt;=[1]Settings!$B$31),[1]Settings!$B$33,0)+IF(AND(G14&lt;[1]Settings!$C$31,(G14+F14)&gt;=[1]Settings!$C$31),[1]Settings!$C$33,0)+IF(AND(G14&lt;[1]Settings!$D$31,(G14+F14)&gt;=[1]Settings!$D$31),[1]Settings!$D$33,0))</f>
+        <v>0</v>
       </c>
       <c r="J14" s="74">
-        <f t="shared" ref="J10:J58" si="2">IF(C14="","",F14+I14)</f>
-        <v>7650</v>
+        <f t="shared" si="2"/>
+        <v>8050</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="19.5" customHeight="1">
@@ -2361,7 +2551,7 @@
         <v/>
       </c>
       <c r="F15" t="str">
-        <f>IF(C15="","",(C15/1000*Settings!$B$16*$H$6)+MAX(0,MIN(G15+(C15/1000*Settings!$B$16*$H$6),Settings!$C$31)-MAX(G15,Settings!$B$31))*Settings!$B$32+MAX(0,MIN(G15+(C15/1000*Settings!$B$16*$H$6),Settings!$D$31)-MAX(G15,Settings!$C$31))*Settings!$C$32+MAX(0,(G15+(C15/1000*Settings!$B$16*$H$6))-MAX(G15,Settings!$D$31))*Settings!$D$32)</f>
+        <f>IF(C15="","",(C15/1000*[1]Settings!$B$16*$H$6)+MAX(0,MIN(G15+(C15/1000*[1]Settings!$B$16*$H$6),[1]Settings!$C$31)-MAX(G15,[1]Settings!$B$31))*[1]Settings!$B$32+MAX(0,MIN(G15+(C15/1000*[1]Settings!$B$16*$H$6),[1]Settings!$D$31)-MAX(G15,[1]Settings!$C$31))*[1]Settings!$C$32+MAX(0,(G15+(C15/1000*[1]Settings!$B$16*$H$6))-MAX(G15,[1]Settings!$D$31))*[1]Settings!$D$32)</f>
         <v/>
       </c>
       <c r="G15" s="73" t="str">
@@ -2369,11 +2559,11 @@
         <v/>
       </c>
       <c r="H15" t="str">
-        <f>IF(OR(C15="",C15=0),"",(F15-(C15/1000*Settings!$B$16*$H$6))/(C15/1000*Settings!$B$16*$H$6))</f>
+        <f>IF(OR(C15="",C15=0),"",(F15-(C15/1000*[1]Settings!$B$16*$H$6))/(C15/1000*[1]Settings!$B$16*$H$6))</f>
         <v/>
       </c>
       <c r="I15" s="72" t="str">
-        <f>IF(C15="","",IF(AND(G15&lt;Settings!$B$31,(G15+F15)&gt;=Settings!$B$31),Settings!$B$33,0)+IF(AND(G15&lt;Settings!$C$31,(G15+F15)&gt;=Settings!$C$31),Settings!$C$33,0)+IF(AND(G15&lt;Settings!$D$31,(G15+F15)&gt;=Settings!$D$31),Settings!$D$33,0))</f>
+        <f>IF(C15="","",IF(AND(G15&lt;[1]Settings!$B$31,(G15+F15)&gt;=[1]Settings!$B$31),[1]Settings!$B$33,0)+IF(AND(G15&lt;[1]Settings!$C$31,(G15+F15)&gt;=[1]Settings!$C$31),[1]Settings!$C$33,0)+IF(AND(G15&lt;[1]Settings!$D$31,(G15+F15)&gt;=[1]Settings!$D$31),[1]Settings!$D$33,0))</f>
         <v/>
       </c>
       <c r="J15" s="74" t="str">
@@ -2388,11 +2578,11 @@
       <c r="B16" s="31"/>
       <c r="C16" s="40"/>
       <c r="D16" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="D14:D40" si="3">IF(C16="","",C16*$E$6)</f>
         <v/>
       </c>
       <c r="E16" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="E14:E40" si="4">IF(C16="","",C16-D16)</f>
         <v/>
       </c>
       <c r="F16" t="str">
@@ -2412,7 +2602,7 @@
         <v/>
       </c>
       <c r="J16" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="J14:J58" si="5">IF(C16="","",F16+I16)</f>
         <v/>
       </c>
     </row>
@@ -2423,11 +2613,11 @@
       <c r="B17" s="31"/>
       <c r="C17" s="40"/>
       <c r="D17" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E17" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F17" t="str">
@@ -2447,7 +2637,7 @@
         <v/>
       </c>
       <c r="J17" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2458,11 +2648,11 @@
       <c r="B18" s="31"/>
       <c r="C18" s="40"/>
       <c r="D18" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E18" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F18" t="str">
@@ -2482,7 +2672,7 @@
         <v/>
       </c>
       <c r="J18" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2493,11 +2683,11 @@
       <c r="B19" s="31"/>
       <c r="C19" s="40"/>
       <c r="D19" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E19" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F19" t="str">
@@ -2517,7 +2707,7 @@
         <v/>
       </c>
       <c r="J19" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2528,11 +2718,11 @@
       <c r="B20" s="31"/>
       <c r="C20" s="40"/>
       <c r="D20" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E20" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F20" t="str">
@@ -2552,7 +2742,7 @@
         <v/>
       </c>
       <c r="J20" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2563,11 +2753,11 @@
       <c r="B21" s="31"/>
       <c r="C21" s="40"/>
       <c r="D21" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E21" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F21" t="str">
@@ -2587,7 +2777,7 @@
         <v/>
       </c>
       <c r="J21" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2598,11 +2788,11 @@
       <c r="B22" s="31"/>
       <c r="C22" s="40"/>
       <c r="D22" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E22" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F22" t="str">
@@ -2622,7 +2812,7 @@
         <v/>
       </c>
       <c r="J22" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2633,11 +2823,11 @@
       <c r="B23" s="31"/>
       <c r="C23" s="40"/>
       <c r="D23" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E23" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F23" t="str">
@@ -2657,7 +2847,7 @@
         <v/>
       </c>
       <c r="J23" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2668,11 +2858,11 @@
       <c r="B24" s="31"/>
       <c r="C24" s="40"/>
       <c r="D24" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E24" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F24" t="str">
@@ -2692,7 +2882,7 @@
         <v/>
       </c>
       <c r="J24" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2703,11 +2893,11 @@
       <c r="B25" s="31"/>
       <c r="C25" s="40"/>
       <c r="D25" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E25" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F25" t="str">
@@ -2727,7 +2917,7 @@
         <v/>
       </c>
       <c r="J25" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2738,11 +2928,11 @@
       <c r="B26" s="31"/>
       <c r="C26" s="40"/>
       <c r="D26" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E26" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F26" t="str">
@@ -2762,7 +2952,7 @@
         <v/>
       </c>
       <c r="J26" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2773,11 +2963,11 @@
       <c r="B27" s="31"/>
       <c r="C27" s="40"/>
       <c r="D27" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E27" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F27" t="str">
@@ -2797,7 +2987,7 @@
         <v/>
       </c>
       <c r="J27" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2808,11 +2998,11 @@
       <c r="B28" s="31"/>
       <c r="C28" s="40"/>
       <c r="D28" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E28" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F28" t="str">
@@ -2832,7 +3022,7 @@
         <v/>
       </c>
       <c r="J28" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2843,11 +3033,11 @@
       <c r="B29" s="31"/>
       <c r="C29" s="40"/>
       <c r="D29" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E29" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F29" t="str">
@@ -2867,7 +3057,7 @@
         <v/>
       </c>
       <c r="J29" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2878,11 +3068,11 @@
       <c r="B30" s="31"/>
       <c r="C30" s="40"/>
       <c r="D30" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E30" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F30" t="str">
@@ -2902,7 +3092,7 @@
         <v/>
       </c>
       <c r="J30" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2913,11 +3103,11 @@
       <c r="B31" s="31"/>
       <c r="C31" s="40"/>
       <c r="D31" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E31" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F31" t="str">
@@ -2937,7 +3127,7 @@
         <v/>
       </c>
       <c r="J31" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2948,11 +3138,11 @@
       <c r="B32" s="31"/>
       <c r="C32" s="40"/>
       <c r="D32" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E32" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F32" t="str">
@@ -2972,7 +3162,7 @@
         <v/>
       </c>
       <c r="J32" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2983,11 +3173,11 @@
       <c r="B33" s="31"/>
       <c r="C33" s="40"/>
       <c r="D33" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E33" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F33" t="str">
@@ -3007,7 +3197,7 @@
         <v/>
       </c>
       <c r="J33" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3018,11 +3208,11 @@
       <c r="B34" s="31"/>
       <c r="C34" s="40"/>
       <c r="D34" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E34" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F34" t="str">
@@ -3042,7 +3232,7 @@
         <v/>
       </c>
       <c r="J34" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3053,11 +3243,11 @@
       <c r="B35" s="31"/>
       <c r="C35" s="40"/>
       <c r="D35" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E35" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F35" t="str">
@@ -3077,7 +3267,7 @@
         <v/>
       </c>
       <c r="J35" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3088,11 +3278,11 @@
       <c r="B36" s="31"/>
       <c r="C36" s="40"/>
       <c r="D36" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E36" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F36" t="str">
@@ -3112,7 +3302,7 @@
         <v/>
       </c>
       <c r="J36" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3123,11 +3313,11 @@
       <c r="B37" s="31"/>
       <c r="C37" s="40"/>
       <c r="D37" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E37" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F37" t="str">
@@ -3147,7 +3337,7 @@
         <v/>
       </c>
       <c r="J37" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3158,11 +3348,11 @@
       <c r="B38" s="31"/>
       <c r="C38" s="40"/>
       <c r="D38" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E38" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F38" t="str">
@@ -3182,7 +3372,7 @@
         <v/>
       </c>
       <c r="J38" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3193,11 +3383,11 @@
       <c r="B39" s="31"/>
       <c r="C39" s="40"/>
       <c r="D39" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E39" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F39" t="str">
@@ -3217,7 +3407,7 @@
         <v/>
       </c>
       <c r="J39" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3228,11 +3418,11 @@
       <c r="B40" s="31"/>
       <c r="C40" s="40"/>
       <c r="D40" s="41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="E40" s="41" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F40" t="str">
@@ -3252,7 +3442,7 @@
         <v/>
       </c>
       <c r="J40" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3263,11 +3453,11 @@
       <c r="B41" s="31"/>
       <c r="C41" s="40"/>
       <c r="D41" s="41" t="str">
-        <f t="shared" ref="D41:D58" si="3">IF(C41="","",C41*$E$6)</f>
+        <f t="shared" ref="D41:D58" si="6">IF(C41="","",C41*$E$6)</f>
         <v/>
       </c>
       <c r="E41" s="41" t="str">
-        <f t="shared" ref="E41:E58" si="4">IF(C41="","",C41-D41)</f>
+        <f t="shared" ref="E41:E58" si="7">IF(C41="","",C41-D41)</f>
         <v/>
       </c>
       <c r="F41" t="str">
@@ -3287,7 +3477,7 @@
         <v/>
       </c>
       <c r="J41" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3298,11 +3488,11 @@
       <c r="B42" s="31"/>
       <c r="C42" s="40"/>
       <c r="D42" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E42" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F42" t="str">
@@ -3322,7 +3512,7 @@
         <v/>
       </c>
       <c r="J42" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3333,11 +3523,11 @@
       <c r="B43" s="31"/>
       <c r="C43" s="40"/>
       <c r="D43" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E43" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F43" t="str">
@@ -3357,7 +3547,7 @@
         <v/>
       </c>
       <c r="J43" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3368,11 +3558,11 @@
       <c r="B44" s="31"/>
       <c r="C44" s="40"/>
       <c r="D44" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E44" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F44" t="str">
@@ -3392,7 +3582,7 @@
         <v/>
       </c>
       <c r="J44" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3403,11 +3593,11 @@
       <c r="B45" s="31"/>
       <c r="C45" s="40"/>
       <c r="D45" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E45" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F45" t="str">
@@ -3427,7 +3617,7 @@
         <v/>
       </c>
       <c r="J45" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3438,11 +3628,11 @@
       <c r="B46" s="31"/>
       <c r="C46" s="40"/>
       <c r="D46" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E46" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F46" t="str">
@@ -3462,7 +3652,7 @@
         <v/>
       </c>
       <c r="J46" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3473,11 +3663,11 @@
       <c r="B47" s="31"/>
       <c r="C47" s="40"/>
       <c r="D47" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E47" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F47" t="str">
@@ -3497,7 +3687,7 @@
         <v/>
       </c>
       <c r="J47" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3508,11 +3698,11 @@
       <c r="B48" s="31"/>
       <c r="C48" s="40"/>
       <c r="D48" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E48" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F48" t="str">
@@ -3532,7 +3722,7 @@
         <v/>
       </c>
       <c r="J48" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3543,11 +3733,11 @@
       <c r="B49" s="31"/>
       <c r="C49" s="40"/>
       <c r="D49" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E49" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F49" t="str">
@@ -3567,7 +3757,7 @@
         <v/>
       </c>
       <c r="J49" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3578,11 +3768,11 @@
       <c r="B50" s="31"/>
       <c r="C50" s="40"/>
       <c r="D50" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E50" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F50" t="str">
@@ -3602,7 +3792,7 @@
         <v/>
       </c>
       <c r="J50" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3613,11 +3803,11 @@
       <c r="B51" s="31"/>
       <c r="C51" s="40"/>
       <c r="D51" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E51" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F51" t="str">
@@ -3637,7 +3827,7 @@
         <v/>
       </c>
       <c r="J51" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3648,11 +3838,11 @@
       <c r="B52" s="31"/>
       <c r="C52" s="40"/>
       <c r="D52" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E52" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F52" t="str">
@@ -3672,7 +3862,7 @@
         <v/>
       </c>
       <c r="J52" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3683,11 +3873,11 @@
       <c r="B53" s="31"/>
       <c r="C53" s="40"/>
       <c r="D53" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E53" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F53" t="str">
@@ -3707,7 +3897,7 @@
         <v/>
       </c>
       <c r="J53" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3718,11 +3908,11 @@
       <c r="B54" s="31"/>
       <c r="C54" s="40"/>
       <c r="D54" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E54" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F54" t="str">
@@ -3742,7 +3932,7 @@
         <v/>
       </c>
       <c r="J54" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3753,11 +3943,11 @@
       <c r="B55" s="31"/>
       <c r="C55" s="40"/>
       <c r="D55" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E55" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F55" t="str">
@@ -3777,7 +3967,7 @@
         <v/>
       </c>
       <c r="J55" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3788,11 +3978,11 @@
       <c r="B56" s="31"/>
       <c r="C56" s="40"/>
       <c r="D56" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E56" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F56" t="str">
@@ -3812,7 +4002,7 @@
         <v/>
       </c>
       <c r="J56" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3823,11 +4013,11 @@
       <c r="B57" s="31"/>
       <c r="C57" s="40"/>
       <c r="D57" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E57" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F57" t="str">
@@ -3847,7 +4037,7 @@
         <v/>
       </c>
       <c r="J57" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3858,11 +4048,11 @@
       <c r="B58" s="31"/>
       <c r="C58" s="40"/>
       <c r="D58" s="41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="E58" s="41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="F58" t="str">
@@ -3882,7 +4072,7 @@
         <v/>
       </c>
       <c r="J58" s="74" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -3893,27 +4083,27 @@
       <c r="B60" s="43"/>
       <c r="C60" s="45">
         <f>SUM(C9:C58)</f>
-        <v>7000000</v>
+        <v>18700000</v>
       </c>
       <c r="D60" s="45">
         <f>SUM(D9:D58)</f>
-        <v>560000</v>
+        <v>1496000</v>
       </c>
       <c r="E60" s="45">
         <f>SUM(E9:E58)</f>
-        <v>6440000</v>
+        <v>17204000</v>
       </c>
       <c r="F60" s="75">
         <f>SUM(F9:F58)</f>
-        <v>7350</v>
+        <v>20676</v>
       </c>
       <c r="I60" s="75">
         <f>SUM(I9:I58)</f>
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="J60" s="75">
         <f>SUM(J9:J58)</f>
-        <v>7650</v>
+        <v>21276</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="15.75">
@@ -3927,7 +4117,7 @@
       </c>
       <c r="B63" s="44">
         <f>C60</f>
-        <v>7000000</v>
+        <v>18700000</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -3985,7 +4175,7 @@
       </c>
       <c r="B76" s="76">
         <f>J60</f>
-        <v>7650</v>
+        <v>21276</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -4003,7 +4193,7 @@
       </c>
       <c r="B78" s="51">
         <f>B76*B77</f>
-        <v>7650</v>
+        <v>21276</v>
       </c>
     </row>
   </sheetData>
@@ -4177,7 +4367,7 @@
       </c>
       <c r="B6" s="57">
         <f>'Bill Calculator'!C60</f>
-        <v>7000000</v>
+        <v>18700000</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="19.5" customHeight="1">
@@ -4186,7 +4376,7 @@
       </c>
       <c r="B7" s="57">
         <f>'Bill Calculator'!D60</f>
-        <v>560000</v>
+        <v>1496000</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="19.5" customHeight="1">
@@ -4195,7 +4385,7 @@
       </c>
       <c r="B8" s="57">
         <f>'Bill Calculator'!E60</f>
-        <v>6440000</v>
+        <v>17204000</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="19.5" customHeight="1">
@@ -4204,7 +4394,7 @@
       </c>
       <c r="B9" s="49">
         <f>'Bill Calculator'!J60</f>
-        <v>7650</v>
+        <v>21276</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="19.5" customHeight="1">
@@ -4213,7 +4403,7 @@
       </c>
       <c r="B10" s="57">
         <f>'Bill Calculator'!B78</f>
-        <v>7650</v>
+        <v>21276</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="19.5" customHeight="1">
@@ -4222,7 +4412,7 @@
       </c>
       <c r="B11" s="58">
         <f>B7+B10</f>
-        <v>567650</v>
+        <v>1517276</v>
       </c>
       <c r="D11" t="s">
         <v>90</v>
@@ -4234,7 +4424,7 @@
       </c>
       <c r="B12" s="59">
         <f>IFERROR(B11/B6,0)</f>
-        <v>8.1092857142857147E-2</v>
+        <v>8.1137754010695187E-2</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="19.5" customHeight="1"/>
@@ -9098,21 +9288,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002CF73862066A8342AF466EC59B30F453" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="74642983bb7c8f2acad9a82d766aed7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f29b6056-a9a8-463d-8257-88e9b79ec5b3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5453f3d78671bba71fc1b1ad2a9e8aab" ns2:_="">
     <xsd:import namespace="f29b6056-a9a8-463d-8257-88e9b79ec5b3"/>
@@ -9250,24 +9425,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A24F8DD5-2CB8-4A1D-A169-13F927CE171C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08878C31-A4B9-45CE-BB5D-9318832972F1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48CD9D30-DEF9-46FB-8357-4BEF32C4BE65}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9283,4 +9456,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08878C31-A4B9-45CE-BB5D-9318832972F1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A24F8DD5-2CB8-4A1D-A169-13F927CE171C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>